<commit_message>
KPI actualizado 2026-08-20 20:43 UTC
</commit_message>
<xml_diff>
--- a/data/50001576-  XEMORTIZ FIRST MAJESTIC.xlsx
+++ b/data/50001576-  XEMORTIZ FIRST MAJESTIC.xlsx
@@ -380,7 +380,7 @@
     <t>Generacion Oc  OT 4375</t>
   </si>
   <si>
-    <t xml:space="preserve">propuesta fabricación externa </t>
+    <t xml:space="preserve">propuesta fabricación externa ,propuesta fabricación externa </t>
   </si>
   <si>
     <t>Armado OT 4375,Fabricación externa  OT 4375</t>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="C31" s="10"/>
       <c r="D31" s="9">
-        <v>46237.55371150463</v>
+        <v>46254.64730673611</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>114</v>

</xml_diff>